<commit_message>
refactor(milestone): finalize specialist services and content cleanup
</commit_message>
<xml_diff>
--- a/design/Lojalność NPC.xlsx
+++ b/design/Lojalność NPC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryczku\Documents\Godmist\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E1E580-348F-471C-98F1-A9ADC7F237FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91A94FC-F5E3-4714-8641-1A9AE1FAEEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,9 +35,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
   <si>
-    <t>Lojalność</t>
-  </si>
-  <si>
     <t>KOWAL</t>
   </si>
   <si>
@@ -156,6 +153,9 @@
   </si>
   <si>
     <t>13 - 41</t>
+  </si>
+  <si>
+    <t>tko ma</t>
   </si>
 </sst>
 </file>
@@ -583,29 +583,29 @@
     <col min="2" max="2" width="65.140625" customWidth="1"/>
     <col min="3" max="3" width="77.140625" customWidth="1"/>
     <col min="4" max="4" width="72.42578125" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" customWidth="1"/>
     <col min="7" max="7" width="68.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -613,17 +613,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="e">
-        <f t="shared" ref="E2:E16" ca="1" si="0">CEILING(POW(4, A2/3+4),1)</f>
-        <v>#NAME?</v>
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <f>ROUNDUP(POWER(4, A2/3+4),0)</f>
+        <v>407</v>
       </c>
       <c r="F2" s="5">
         <f>0</f>
@@ -635,21 +635,21 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F3" s="5" t="e">
-        <f ca="1">SUM(E2)</f>
-        <v>#NAME?</v>
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E16" si="0">ROUNDUP(POWER(4, A3/3+4),0)</f>
+        <v>646</v>
+      </c>
+      <c r="F3" s="5">
+        <f>SUM(E2)</f>
+        <v>407</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -657,21 +657,21 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F4" s="5" t="e">
-        <f t="shared" ref="F4:F17" ca="1" si="1">SUM($E$2:E3)</f>
-        <v>#NAME?</v>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>1024</v>
+      </c>
+      <c r="F4" s="5">
+        <f t="shared" ref="F4:F17" si="1">SUM($E$2:E3)</f>
+        <v>1053</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -679,21 +679,21 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F5" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>1626</v>
+      </c>
+      <c r="F5" s="5">
+        <f t="shared" si="1"/>
+        <v>2077</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -701,21 +701,21 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F6" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>2581</v>
+      </c>
+      <c r="F6" s="5">
+        <f t="shared" si="1"/>
+        <v>3703</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -723,21 +723,21 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F7" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>4096</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" si="1"/>
+        <v>6284</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -745,21 +745,21 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F8" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>15</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>6502</v>
+      </c>
+      <c r="F8" s="5">
+        <f t="shared" si="1"/>
+        <v>10380</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -767,21 +767,21 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F9" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>10322</v>
+      </c>
+      <c r="F9" s="5">
+        <f t="shared" si="1"/>
+        <v>16882</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -789,21 +789,21 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F10" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>18</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>16384</v>
+      </c>
+      <c r="F10" s="5">
+        <f t="shared" si="1"/>
+        <v>27204</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -811,21 +811,21 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F11" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>19</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>26008</v>
+      </c>
+      <c r="F11" s="5">
+        <f t="shared" si="1"/>
+        <v>43588</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -833,21 +833,21 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F12" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>41286</v>
+      </c>
+      <c r="F12" s="5">
+        <f t="shared" si="1"/>
+        <v>69596</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -855,21 +855,21 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F13" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>23</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>65536</v>
+      </c>
+      <c r="F13" s="5">
+        <f t="shared" si="1"/>
+        <v>110882</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -877,21 +877,21 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F14" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+        <v>24</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>104032</v>
+      </c>
+      <c r="F14" s="5">
+        <f t="shared" si="1"/>
+        <v>176418</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -899,21 +899,21 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F15" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>165141</v>
+      </c>
+      <c r="F15" s="5">
+        <f t="shared" si="1"/>
+        <v>280450</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -921,45 +921,45 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="F16" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>262144</v>
+      </c>
+      <c r="F16" s="5">
+        <f t="shared" si="1"/>
+        <v>445591</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="C17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="D17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F17" s="5" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="F17" s="5">
+        <f t="shared" si="1"/>
+        <v>707735</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18" s="10"/>
       <c r="F18" s="5"/>
@@ -967,7 +967,7 @@
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D19" s="10"/>
       <c r="F19" s="3"/>
@@ -975,20 +975,20 @@
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F22" s="5"/>
     </row>

</xml_diff>